<commit_message>
els and enrico comments
</commit_message>
<xml_diff>
--- a/rules/CORE-000238/negative/01/data/unit-test-coreid-CG0147-negative 1.xlsx
+++ b/rules/CORE-000238/negative/01/data/unit-test-coreid-CG0147-negative 1.xlsx
@@ -160,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -177,6 +177,7 @@
     <xf numFmtId="0" fontId="12" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -667,7 +668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -946,6 +947,85 @@
       <c r="F10" t="inlineStr">
         <is>
           <t>2014-01-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>dm.xpt</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>8</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>RFXENDTC</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2014-01-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ex.xpt</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>65</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>$max_ex_exstdtc</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2014-01-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ex.xpt</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>65</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>$max_ex_exendtc</t>
         </is>
       </c>
     </row>
@@ -960,7 +1040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z7"/>
+  <dimension ref="A1:Z8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1760,6 +1840,116 @@
         </is>
       </c>
       <c r="Z7" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CDISCPILOT01</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>GUARD-NO-EXEN</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1115</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2012-11-30</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2013-01-23</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2014-01-01</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>2014-01-15</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2012-11-23</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2013-05-20</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>1928</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>84</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>YEARS</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>WHITE</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>NOT HISPANIC OR LATINO</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>ZAN_LOW</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Zanomaline Low Dose (54 mg)</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>ZAN_LOW</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Zanomaline Low Dose (54 mg)</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
@@ -1776,7 +1966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q63"/>
+  <dimension ref="A1:Q65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6754,6 +6944,154 @@
         <v>1</v>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>CDISCPILOT01</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>GUARD-NO-EXEN</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>DEV0001</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>1</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>ZANOMALINE</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>54</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>INJECTION</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>QD</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>SUBCUTANEOUS</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>SDS580-359</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>TREATMENT</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>2014-01-01</t>
+        </is>
+      </c>
+      <c r="P64" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>CDISCPILOT01</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>GUARD-NO-EXEN</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>DEV0001</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>2</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>ZANOMALINE</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>54</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>INJECTION</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>QD</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>SUBCUTANEOUS</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>SDS580-359</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>TREATMENT</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>2014-01-10</t>
+        </is>
+      </c>
+      <c r="P65" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>